<commit_message>
Write nullable numbers as numbers
</commit_message>
<xml_diff>
--- a/src/Excelsior.Tests/BannerTests.ExpandsHeightForMultilineText.verified.xlsx
+++ b/src/Excelsior.Tests/BannerTests.ExpandsHeightForMultilineText.verified.xlsx
@@ -256,7 +256,7 @@
       <formula>LEN(TRIM(C3))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="6">
+  <dataValidations count="7">
     <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a number." prompt="Required field" sqref="A3:A6">
       <formula1>ISNUMBER(A3)</formula1>
     </dataValidation>
@@ -265,6 +265,10 @@
     </dataValidation>
     <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="This field is required." prompt="Required field" sqref="C3:C6">
       <formula1>LEN(TRIM(C3))&gt;0</formula1>
+    </dataValidation>
+    <dataValidation type="date" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a valid date.&#10;yyyy-MM-dd" prompt="Date as yyyy-MM-dd" sqref="D3:D6">
+      <formula1>2</formula1>
+      <formula2>2958465</formula2>
     </dataValidation>
     <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a number." sqref="E3:E6">
       <formula1>ISNUMBER(E3)</formula1>

</xml_diff>

<commit_message>
Write nullable numbers as numbers (#258)
</commit_message>
<xml_diff>
--- a/src/Excelsior.Tests/BannerTests.ExpandsHeightForMultilineText.verified.xlsx
+++ b/src/Excelsior.Tests/BannerTests.ExpandsHeightForMultilineText.verified.xlsx
@@ -256,7 +256,7 @@
       <formula>LEN(TRIM(C3))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="6">
+  <dataValidations count="7">
     <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a number." prompt="Required field" sqref="A3:A6">
       <formula1>ISNUMBER(A3)</formula1>
     </dataValidation>
@@ -265,6 +265,10 @@
     </dataValidation>
     <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="This field is required." prompt="Required field" sqref="C3:C6">
       <formula1>LEN(TRIM(C3))&gt;0</formula1>
+    </dataValidation>
+    <dataValidation type="date" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a valid date.&#10;yyyy-MM-dd" prompt="Date as yyyy-MM-dd" sqref="D3:D6">
+      <formula1>2</formula1>
+      <formula2>2958465</formula2>
     </dataValidation>
     <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a number." sqref="E3:E6">
       <formula1>ISNUMBER(E3)</formula1>

</xml_diff>